<commit_message>
Updated locus export after schema update
</commit_message>
<xml_diff>
--- a/tabular/sublineage/herv_sublineage_ltr_data_all.xlsx
+++ b/tabular/sublineage/herv_sublineage_ltr_data_all.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/erv/locus-level/ERVdb-HomoSapiens/tabular/sublineage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C708C70E-DD6C-F54B-91D1-ECF75CC54BC4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA84785D-E1C4-2F4D-9740-73FDCE855107}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="720" windowWidth="21060" windowHeight="16940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7200" yWindow="720" windowWidth="21060" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ltr_lineage_table" sheetId="1" r:id="rId1"/>
@@ -2132,7 +2132,7 @@
         <v>4</v>
       </c>
       <c r="I11" t="str">
-        <f>IF(A11&lt;&gt;B11,"FLAG","")</f>
+        <f t="shared" ref="I11:I42" si="0">IF(A11&lt;&gt;B11,"FLAG","")</f>
         <v/>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
         <v>4</v>
       </c>
       <c r="I12" t="str">
-        <f>IF(A12&lt;&gt;B12,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2192,7 +2192,7 @@
         <v>4</v>
       </c>
       <c r="I13" t="str">
-        <f>IF(A13&lt;&gt;B13,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2222,7 +2222,7 @@
         <v>4</v>
       </c>
       <c r="I14" t="str">
-        <f>IF(A14&lt;&gt;B14,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2252,7 +2252,7 @@
         <v>4</v>
       </c>
       <c r="I15" t="str">
-        <f>IF(A15&lt;&gt;B15,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2282,7 +2282,7 @@
         <v>4</v>
       </c>
       <c r="I16" t="str">
-        <f>IF(A16&lt;&gt;B16,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2312,7 +2312,7 @@
         <v>4</v>
       </c>
       <c r="I17" t="str">
-        <f>IF(A17&lt;&gt;B17,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2342,7 +2342,7 @@
         <v>4</v>
       </c>
       <c r="I18" t="str">
-        <f>IF(A18&lt;&gt;B18,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
         <v>4</v>
       </c>
       <c r="I19" t="str">
-        <f>IF(A19&lt;&gt;B19,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2402,7 +2402,7 @@
         <v>4</v>
       </c>
       <c r="I20" t="str">
-        <f>IF(A20&lt;&gt;B20,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2432,7 +2432,7 @@
         <v>4</v>
       </c>
       <c r="I21" t="str">
-        <f>IF(A21&lt;&gt;B21,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
         <v>4</v>
       </c>
       <c r="I22" t="str">
-        <f>IF(A22&lt;&gt;B22,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
         <v>4</v>
       </c>
       <c r="I23" t="str">
-        <f>IF(A23&lt;&gt;B23,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2522,7 +2522,7 @@
         <v>4</v>
       </c>
       <c r="I24" t="str">
-        <f>IF(A24&lt;&gt;B24,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2552,7 +2552,7 @@
         <v>4</v>
       </c>
       <c r="I25" t="str">
-        <f>IF(A25&lt;&gt;B25,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2582,7 +2582,7 @@
         <v>4</v>
       </c>
       <c r="I26" t="str">
-        <f>IF(A26&lt;&gt;B26,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
         <v>4</v>
       </c>
       <c r="I27" t="str">
-        <f>IF(A27&lt;&gt;B27,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2642,7 +2642,7 @@
         <v>4</v>
       </c>
       <c r="I28" t="str">
-        <f>IF(A28&lt;&gt;B28,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2672,7 +2672,7 @@
         <v>4</v>
       </c>
       <c r="I29" t="str">
-        <f>IF(A29&lt;&gt;B29,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2702,7 +2702,7 @@
         <v>4</v>
       </c>
       <c r="I30" t="str">
-        <f>IF(A30&lt;&gt;B30,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
         <v>4</v>
       </c>
       <c r="I31" t="str">
-        <f>IF(A31&lt;&gt;B31,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2762,7 +2762,7 @@
         <v>4</v>
       </c>
       <c r="I32" t="str">
-        <f>IF(A32&lt;&gt;B32,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
         <v>4</v>
       </c>
       <c r="I33" t="str">
-        <f>IF(A33&lt;&gt;B33,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
         <v>4</v>
       </c>
       <c r="I34" t="str">
-        <f>IF(A34&lt;&gt;B34,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
         <v>4</v>
       </c>
       <c r="I35" t="str">
-        <f>IF(A35&lt;&gt;B35,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
         <v>4</v>
       </c>
       <c r="I36" t="str">
-        <f>IF(A36&lt;&gt;B36,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
         <v>4</v>
       </c>
       <c r="I37" t="str">
-        <f>IF(A37&lt;&gt;B37,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
         <v>4</v>
       </c>
       <c r="I38" t="str">
-        <f>IF(A38&lt;&gt;B38,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
         <v>4</v>
       </c>
       <c r="I39" t="str">
-        <f>IF(A39&lt;&gt;B39,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
         <v>56</v>
       </c>
       <c r="I40" t="str">
-        <f>IF(A40&lt;&gt;B40,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v>FLAG</v>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
         <v>56</v>
       </c>
       <c r="I41" t="str">
-        <f>IF(A41&lt;&gt;B41,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v>FLAG</v>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
         <v>56</v>
       </c>
       <c r="I42" t="str">
-        <f>IF(A42&lt;&gt;B42,"FLAG","")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
         <v>56</v>
       </c>
       <c r="I43" t="str">
-        <f>IF(A43&lt;&gt;B43,"FLAG","")</f>
+        <f t="shared" ref="I43:I74" si="1">IF(A43&lt;&gt;B43,"FLAG","")</f>
         <v/>
       </c>
     </row>
@@ -3122,7 +3122,7 @@
         <v>56</v>
       </c>
       <c r="I44" t="str">
-        <f>IF(A44&lt;&gt;B44,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3152,7 +3152,7 @@
         <v>56</v>
       </c>
       <c r="I45" t="str">
-        <f>IF(A45&lt;&gt;B45,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3182,7 +3182,7 @@
         <v>4</v>
       </c>
       <c r="I46" t="str">
-        <f>IF(A46&lt;&gt;B46,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3212,7 +3212,7 @@
         <v>4</v>
       </c>
       <c r="I47" t="str">
-        <f>IF(A47&lt;&gt;B47,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3242,7 +3242,7 @@
         <v>4</v>
       </c>
       <c r="I48" t="str">
-        <f>IF(A48&lt;&gt;B48,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3272,7 +3272,7 @@
         <v>4</v>
       </c>
       <c r="I49" t="str">
-        <f>IF(A49&lt;&gt;B49,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3302,7 +3302,7 @@
         <v>4</v>
       </c>
       <c r="I50" t="str">
-        <f>IF(A50&lt;&gt;B50,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3332,7 +3332,7 @@
         <v>4</v>
       </c>
       <c r="I51" t="str">
-        <f>IF(A51&lt;&gt;B51,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3362,7 +3362,7 @@
         <v>4</v>
       </c>
       <c r="I52" t="str">
-        <f>IF(A52&lt;&gt;B52,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
         <v>4</v>
       </c>
       <c r="I53" t="str">
-        <f>IF(A53&lt;&gt;B53,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3422,7 +3422,7 @@
         <v>4</v>
       </c>
       <c r="I54" t="str">
-        <f>IF(A54&lt;&gt;B54,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3452,7 +3452,7 @@
         <v>4</v>
       </c>
       <c r="I55" t="str">
-        <f>IF(A55&lt;&gt;B55,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
         <v>4</v>
       </c>
       <c r="I56" t="str">
-        <f>IF(A56&lt;&gt;B56,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3512,7 +3512,7 @@
         <v>4</v>
       </c>
       <c r="I57" t="str">
-        <f>IF(A57&lt;&gt;B57,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3542,7 +3542,7 @@
         <v>4</v>
       </c>
       <c r="I58" t="str">
-        <f>IF(A58&lt;&gt;B58,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
         <v>4</v>
       </c>
       <c r="I59" t="str">
-        <f>IF(A59&lt;&gt;B59,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3602,7 +3602,7 @@
         <v>4</v>
       </c>
       <c r="I60" t="str">
-        <f>IF(A60&lt;&gt;B60,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3632,7 +3632,7 @@
         <v>4</v>
       </c>
       <c r="I61" t="str">
-        <f>IF(A61&lt;&gt;B61,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3662,7 +3662,7 @@
         <v>4</v>
       </c>
       <c r="I62" t="str">
-        <f>IF(A62&lt;&gt;B62,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3692,7 +3692,7 @@
         <v>4</v>
       </c>
       <c r="I63" t="str">
-        <f>IF(A63&lt;&gt;B63,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
         <v>4</v>
       </c>
       <c r="I64" t="str">
-        <f>IF(A64&lt;&gt;B64,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3752,7 +3752,7 @@
         <v>4</v>
       </c>
       <c r="I65" t="str">
-        <f>IF(A65&lt;&gt;B65,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3782,7 +3782,7 @@
         <v>4</v>
       </c>
       <c r="I66" t="str">
-        <f>IF(A66&lt;&gt;B66,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
         <v>4</v>
       </c>
       <c r="I67" t="str">
-        <f>IF(A67&lt;&gt;B67,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3842,7 +3842,7 @@
         <v>4</v>
       </c>
       <c r="I68" t="str">
-        <f>IF(A68&lt;&gt;B68,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3872,7 +3872,7 @@
         <v>4</v>
       </c>
       <c r="I69" t="str">
-        <f>IF(A69&lt;&gt;B69,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3902,7 +3902,7 @@
         <v>4</v>
       </c>
       <c r="I70" t="str">
-        <f>IF(A70&lt;&gt;B70,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
         <v>4</v>
       </c>
       <c r="I71" t="str">
-        <f>IF(A71&lt;&gt;B71,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
         <v>4</v>
       </c>
       <c r="I72" t="str">
-        <f>IF(A72&lt;&gt;B72,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -3992,7 +3992,7 @@
         <v>4</v>
       </c>
       <c r="I73" t="str">
-        <f>IF(A73&lt;&gt;B73,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
         <v>4</v>
       </c>
       <c r="I74" t="str">
-        <f>IF(A74&lt;&gt;B74,"FLAG","")</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -4052,7 +4052,7 @@
         <v>4</v>
       </c>
       <c r="I75" t="str">
-        <f>IF(A75&lt;&gt;B75,"FLAG","")</f>
+        <f t="shared" ref="I75:I91" si="2">IF(A75&lt;&gt;B75,"FLAG","")</f>
         <v/>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
         <v>4</v>
       </c>
       <c r="I76" t="str">
-        <f>IF(A76&lt;&gt;B76,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4112,7 +4112,7 @@
         <v>4</v>
       </c>
       <c r="I77" t="str">
-        <f>IF(A77&lt;&gt;B77,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
         <v>4</v>
       </c>
       <c r="I78" t="str">
-        <f>IF(A78&lt;&gt;B78,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4172,7 +4172,7 @@
         <v>4</v>
       </c>
       <c r="I79" t="str">
-        <f>IF(A79&lt;&gt;B79,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
         <v>4</v>
       </c>
       <c r="I80" t="str">
-        <f>IF(A80&lt;&gt;B80,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4232,7 +4232,7 @@
         <v>4</v>
       </c>
       <c r="I81" t="str">
-        <f>IF(A81&lt;&gt;B81,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4262,7 +4262,7 @@
         <v>4</v>
       </c>
       <c r="I82" t="str">
-        <f>IF(A82&lt;&gt;B82,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
         <v>4</v>
       </c>
       <c r="I83" t="str">
-        <f>IF(A83&lt;&gt;B83,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4322,7 +4322,7 @@
         <v>4</v>
       </c>
       <c r="I84" t="str">
-        <f>IF(A84&lt;&gt;B84,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4352,7 +4352,7 @@
         <v>4</v>
       </c>
       <c r="I85" t="str">
-        <f>IF(A85&lt;&gt;B85,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4382,7 +4382,7 @@
         <v>4</v>
       </c>
       <c r="I86" t="str">
-        <f>IF(A86&lt;&gt;B86,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4412,7 +4412,7 @@
         <v>4</v>
       </c>
       <c r="I87" t="str">
-        <f>IF(A87&lt;&gt;B87,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4442,7 +4442,7 @@
         <v>4</v>
       </c>
       <c r="I88" t="str">
-        <f>IF(A88&lt;&gt;B88,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
         <v>4</v>
       </c>
       <c r="I89" t="str">
-        <f>IF(A89&lt;&gt;B89,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
         <v>4</v>
       </c>
       <c r="I90" t="str">
-        <f>IF(A90&lt;&gt;B90,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4532,7 +4532,7 @@
         <v>4</v>
       </c>
       <c r="I91" t="str">
-        <f>IF(A91&lt;&gt;B91,"FLAG","")</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
         <v>4</v>
       </c>
       <c r="I99" t="str">
-        <f>IF(A99&lt;&gt;B99,"FLAG","")</f>
+        <f t="shared" ref="I99:I126" si="3">IF(A99&lt;&gt;B99,"FLAG","")</f>
         <v/>
       </c>
     </row>
@@ -4774,7 +4774,7 @@
         <v>4</v>
       </c>
       <c r="I100" t="str">
-        <f>IF(A100&lt;&gt;B100,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4804,7 +4804,7 @@
         <v>4</v>
       </c>
       <c r="I101" t="str">
-        <f>IF(A101&lt;&gt;B101,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4834,7 +4834,7 @@
         <v>4</v>
       </c>
       <c r="I102" t="str">
-        <f>IF(A102&lt;&gt;B102,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
         <v>4</v>
       </c>
       <c r="I103" t="str">
-        <f>IF(A103&lt;&gt;B103,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4894,7 +4894,7 @@
         <v>4</v>
       </c>
       <c r="I104" t="str">
-        <f>IF(A104&lt;&gt;B104,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
         <v>4</v>
       </c>
       <c r="I105" t="str">
-        <f>IF(A105&lt;&gt;B105,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
         <v>4</v>
       </c>
       <c r="I106" t="str">
-        <f>IF(A106&lt;&gt;B106,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -4984,7 +4984,7 @@
         <v>4</v>
       </c>
       <c r="I107" t="str">
-        <f>IF(A107&lt;&gt;B107,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5014,7 +5014,7 @@
         <v>4</v>
       </c>
       <c r="I108" t="str">
-        <f>IF(A108&lt;&gt;B108,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5044,7 +5044,7 @@
         <v>4</v>
       </c>
       <c r="I109" t="str">
-        <f>IF(A109&lt;&gt;B109,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5074,7 +5074,7 @@
         <v>4</v>
       </c>
       <c r="I110" t="str">
-        <f>IF(A110&lt;&gt;B110,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5104,7 +5104,7 @@
         <v>4</v>
       </c>
       <c r="I111" t="str">
-        <f>IF(A111&lt;&gt;B111,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5134,7 +5134,7 @@
         <v>4</v>
       </c>
       <c r="I112" t="str">
-        <f>IF(A112&lt;&gt;B112,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5164,7 +5164,7 @@
         <v>4</v>
       </c>
       <c r="I113" t="str">
-        <f>IF(A113&lt;&gt;B113,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5194,7 +5194,7 @@
         <v>4</v>
       </c>
       <c r="I114" t="str">
-        <f>IF(A114&lt;&gt;B114,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v>FLAG</v>
       </c>
     </row>
@@ -5224,7 +5224,7 @@
         <v>4</v>
       </c>
       <c r="I115" t="str">
-        <f>IF(A115&lt;&gt;B115,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5254,7 +5254,7 @@
         <v>4</v>
       </c>
       <c r="I116" t="str">
-        <f>IF(A116&lt;&gt;B116,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5284,7 +5284,7 @@
         <v>4</v>
       </c>
       <c r="I117" t="str">
-        <f>IF(A117&lt;&gt;B117,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5314,7 +5314,7 @@
         <v>4</v>
       </c>
       <c r="I118" t="str">
-        <f>IF(A118&lt;&gt;B118,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5344,7 +5344,7 @@
         <v>4</v>
       </c>
       <c r="I119" t="str">
-        <f>IF(A119&lt;&gt;B119,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5374,7 +5374,7 @@
         <v>4</v>
       </c>
       <c r="I120" t="str">
-        <f>IF(A120&lt;&gt;B120,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5404,7 +5404,7 @@
         <v>4</v>
       </c>
       <c r="I121" t="str">
-        <f>IF(A121&lt;&gt;B121,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
         <v>4</v>
       </c>
       <c r="I122" t="str">
-        <f>IF(A122&lt;&gt;B122,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5464,7 +5464,7 @@
         <v>4</v>
       </c>
       <c r="I123" t="str">
-        <f>IF(A123&lt;&gt;B123,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5494,7 +5494,7 @@
         <v>4</v>
       </c>
       <c r="I124" t="str">
-        <f>IF(A124&lt;&gt;B124,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
         <v>4</v>
       </c>
       <c r="I125" t="str">
-        <f>IF(A125&lt;&gt;B125,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -5554,7 +5554,7 @@
         <v>4</v>
       </c>
       <c r="I126" t="str">
-        <f>IF(A126&lt;&gt;B126,"FLAG","")</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>

</xml_diff>